<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.002-03 Victorino souffle au jardin
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.002-03.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.002-03.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le château de terre de Victorina</t>
+          <t>Victorino souffle au jardin</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin</t>
+          <t>jardin, château de terre, pots, terre, bord, soleil, ombre, poussière, fourmi, basilic</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorina, papa, maman</t>
+          <t>Victorino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut un château de terre. Il s'effondre. Elle souffle, fait une pause, puis pose une feuille dessus.</t>
+          <t>Les pots tièdes font une ombre étroite. Près du bord, un éclat de pot brille. Victorino veut le château, maintenant. La terre trop vite, le château s'effondre. Sourire parti, poitrine trop vite, papa accroupi. Il souffle, pause. Merci vécu. Pot trop vite, terre qui glisse. Il s'arrête, lit l'éclat. Un éclat de pot tient sur la terre.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>L'arrosoir penche encore, près des pots. Une goutte tombe dans la terre tiède. Elle fait un petit rond sombre. Un linge blanc bouge sur le fil. Une abeille passe, tout près. Ça sent la terre mouillée. Ça sent aussi le linge au soleil. J'ai arrosé les fleurs, tout doux. La fenêtre est ouverte. J'entends le jardin. La planche est sèche, près des pots. Je veux un château, papa. Un château de terre. Quelle idée. Tes mains peuvent prendre la terre. En ce moment, Victorina est accroupie. Ses mains prennent la terre fraîche. La terre est froide et un peu collante. Elle forme un mur. Puis une tour. Tu appuies tout doucement ? Oui. Un grand château. Le château grandit. Un mur glisse. Le château s'effondre. La terre retombe en tas. Victorina sent sa poitrine aller vite. Ses joues chauffent. Ses épaules se serrent. C'est trop. Je suis fâchée. Le château est tombé. Tu es fâchée. Tu peux souffler. Tu peux faire une pause. Je viens près de la planche. On est ensemble. Victorina s'assoit sur la planche. Elle pose les mains sur ses genoux. Elle souffle comme le vent. Une fois. Deux fois. Elle fait une pause. Le jardin redevient calme. Le linge bouge encore, tout léger. Je souffle. Je fais une pause. Bravo. Ton corps ralentit. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Tout doucement. Victorina reprend une poignée de terre. Elle construit un petit mur. Le château est petit. Il tient.</t>
+          <t>Les pots tièdes font une ombre étroite. Ça sent la terre chaude, un peu. Ça sent bon, papa. Tu la sens, la terre, Victorino ? Oui, papa. Un rayon glisse sur un bord fêlé. Il brille, maman. Le pot est chaud ? Un peu, maman. Le château va commencer. La terre et les pots, d'accord ? Oui, maman. Une fourmi avance le long du bord. Elle marche, papa. Tu la vois, la fourmi ? Oui. La terre est sèche contre la peau. Elle pique, maman. Tu la sens, la terre ? Oui. Près du bord, un éclat de pot brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus des pots. Elle vole, maman. Au-dessus du bord ? Oui, au-dessus. Papa pose les mains près de la terre. La terre est un peu lourde. On fait le château, papa ? Papa prend un peu de terre. Un mur tombe un peu. C'est marron, papa. Comme une maison ? Oui, comme une maison. En ce moment, Victorino tire la terre vers les pots. Je veux le château, maintenant ! Le château, tout de suite. Tu vois la terre, Victorino ? Oui, papa. Victorino ouvre les mains trop vite. Il presse la terre trop fort. Les murs collent trop près. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sa poitrine va trop vite. Ça tombe, Victorino ? Oui, papa. Tes lèvres sont serrées, Victorino ? Un peu, maman. L'éclat de pot tremble, puis tient. Le château s'effondre en tas. C'est trop, papa. Papa s'accroupit à la même hauteur. Victorino regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>L'arrosoir penche encore, près des pots. Une goutte tombe dans la terre tiède. Elle fait un petit rond sombre. Un linge blanc bouge sur le fil. Une abeille passe, tout près. Ça sent la terre mouillée. Ça sent aussi le linge au soleil. J'ai arrosé les fleurs, tout doux. La fenêtre est ouverte. J'entends le jardin. La planche est sèche, près des pots. Je veux un château, papa. Un château de terre. Quelle idée. Tes mains peuvent prendre la terre. En ce moment, Victorina est accroupie. Ses mains prennent la terre fraîche. La terre est froide et un peu collante. Elle forme un mur. Puis une tour. Tu appuies tout doucement ? Oui. Un grand château. Le château grandit. Un mur glisse. Le château s'effondre. La terre retombe en tas. Victorina sent sa poitrine aller vite. Ses joues chauffent. Ses épaules se serrent. C'est trop. Je suis fâchée. Le château est tombé. Tu es fâchée. Tu peux souffler. Tu peux faire une pause. Je viens près de la planche. On est ensemble. Victorina s'assoit sur la planche. Elle pose les mains sur ses genoux. Elle souffle comme le vent. Une fois. Deux fois. Elle fait une pause. Le jardin redevient calme. Le linge bouge encore, tout léger. Je souffle. Je fais une pause. Bravo. Ton corps ralentit. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Tout doucement. Victorina reprend une poignée de terre. Elle construit un petit mur. Le château est petit. Il tient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les pots tièdes font une ombre étroite. Ça sent la terre chaude, un peu. Ça sent bon, papa. Tu la sens, la terre, Victorino ? Oui, papa. Un rayon glisse sur un bord fêlé. Il brille, maman. Le pot est chaud ? Un peu, maman. Le château va commencer. La terre et les pots, d'accord ? Oui, maman. Une fourmi avance le long du bord. Elle marche, papa. Tu la vois, la fourmi ? Oui. La terre est sèche contre la peau. Elle pique, maman. Tu la sens, la terre ? Oui. Près du bord, un &lt;emphasis level="moderate"&gt;éclat de pot&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus des pots. Elle vole, maman. Au-dessus du bord ? Oui, au-dessus. Papa pose les mains près de la terre. La terre est un peu lourde. On fait le château, papa ? Papa prend un peu de terre. Un mur tombe un peu. C'est marron, papa. Comme une maison ? Oui, comme une maison. En ce moment, Victorino tire la terre vers les pots. Je veux le château, maintenant ! Le château, tout de suite. Tu vois la terre, Victorino ? Oui, papa. Victorino ouvre les mains trop vite. Il presse la terre trop fort. Les murs collent trop près. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sa poitrine va trop vite. Ça tombe, Victorino ? Oui, papa. Tes lèvres sont serrées, Victorino ? Un peu, maman. L'éclat de pot tremble, puis tient. Le château s'effondre en tas. C'est trop, papa. Papa s'accroupit à la même hauteur. Victorino regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>William construit un château de terre au jardin. Le château s'effondre. William sent sa poitrine aller vite. Papa est là, près des pots. Papa dit : tu peux &lt;emphasis&gt;souffler&lt;/emphasis&gt;. Tu peux faire une pause. William s'assoit sur la planche. Il souffle comme le vent. Une fois. Deux fois. Il fait une pause. Ses mains se posent sur ses genoux. Le jardin redevient calme. William reprend une poignée de terre. Il construit tout doucement. Papa reste près de lui. Souffler, puis une pause. Puis on reprend. [pause]</t>
+          <t>Les pots tièdes font une ombre étroite. Ça sent la terre chaude, un peu. Ça sent bon, papa. Tu la sens, la terre, Victorino ? Oui, papa. Un rayon glisse sur un bord fêlé. Il brille, maman. Le pot est chaud ? Un peu, maman. Le château va commencer. La terre et les pots, d'accord ? Oui, maman. Une fourmi avance le long du bord. Elle marche, papa. Tu la vois, la fourmi ? Oui. La terre est sèche contre la peau. Elle pique, maman. Tu la sens, la terre ? Oui. Près du bord, un &lt;emphasis&gt;éclat de pot&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus des pots. Elle vole, maman. Au-dessus du bord ? Oui, au-dessus. Papa pose les mains près de la terre. La terre est un peu lourde. On fait le château, papa ? Papa prend un peu de terre. Un mur tombe un peu. C'est marron, papa. Comme une maison ? Oui, comme une maison. En ce moment, Victorino tire la terre vers les pots. Je veux le château, maintenant ! Le château, tout de suite. Tu vois la terre, Victorino ? Oui, papa. Victorino ouvre les mains trop vite. Il presse la terre trop fort. Les murs collent trop près. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sa poitrine va trop vite. Ça tombe, Victorino ? Oui, papa. Tes lèvres sont serrées, Victorino ? Un peu, maman. L'éclat de pot tremble, puis tient. Le château s'effondre en tas. C'est trop, papa. Papa s'accroupit à la même hauteur. Victorino regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>souffler</t>
+          <t>éclat de pot</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,58 +1321,70 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis gêne; intensite=2; destinataire=enfant; sous_texte=il_veut_le_chateau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|L'arrosoir penche encore, près des pots.
-narrateur|Une goutte tombe dans la terre tiède.
-narrateur|Elle fait un petit rond sombre.
-narrateur|Un linge blanc bouge sur le fil.
-narrateur|Une abeille passe, tout près.
-narrateur|Ça sent la terre mouillée.
-narrateur|Ça sent aussi le linge au soleil.
-papa|J'ai arrosé les fleurs, tout doux.
-maman|La fenêtre est ouverte. J'entends le jardin.
-papa|La planche est sèche, près des pots.
-enfant-f|Je veux un château, papa.
-maman|Un château de terre. Quelle idée.
-papa|Tes mains peuvent prendre la terre.
-narrateur|En ce moment, Victorina est accroupie.
-narrateur|Ses mains prennent la terre fraîche.
-narrateur|La terre est froide et un peu collante.
-narrateur|Elle forme un mur.
-narrateur|Puis une tour.
-papa|Tu appuies tout doucement ?
-enfant-f|Oui. Un grand château.
-narrateur|Le château grandit.
-narrateur|Un mur glisse.
-narrateur|Le château s'effondre.
-narrateur|La terre retombe en tas.
-narrateur|Victorina sent sa poitrine aller vite.
-narrateur|Ses joues chauffent.
-narrateur|Ses épaules se serrent.
-enfant-f|C'est trop. Je suis fâchée.
-papa|Le château est tombé. Tu es fâchée.
-papa|Tu peux souffler.
-papa|Tu peux faire une pause.
-maman|Je viens près de la planche. On est ensemble.
-narrateur|Victorina s'assoit sur la planche.
-narrateur|Elle pose les mains sur ses genoux.
-narrateur|Elle souffle comme le vent.
-narrateur|Une fois.
-narrateur|Deux fois.
-narrateur|Elle fait une pause.
-narrateur|Le jardin redevient calme.
-narrateur|Le linge bouge encore, tout léger.
-enfant-f|Je souffle. Je fais une pause.
-maman|Bravo. Ton corps ralentit.
-papa|Tu as soufflé. Tu as fait une pause.
-papa|Tu veux reprendre, tout doucement ?
-enfant-f|Oui. Tout doucement.
-narrateur|Victorina reprend une poignée de terre.
-narrateur|Elle construit un petit mur.
-narrateur|Le château est petit.
-narrateur|Il tient.</t>
+          <t>narrateur|Les pots tièdes font une ombre étroite.
+narrateur|Ça sent la terre chaude, un peu.
+enfant-m|Ça sent bon, papa.
+papa|Tu la sens, la terre, Victorino ?
+enfant-m|Oui, papa.
+narrateur|Un rayon glisse sur un bord fêlé.
+enfant-m|Il brille, maman.
+maman|Le pot est chaud ?
+enfant-m|Un peu, maman.
+maman|Le château va commencer.
+maman|La terre et les pots, d'accord ?
+enfant-m|Oui, maman.
+narrateur|Une fourmi avance le long du bord.
+enfant-m|Elle marche, papa.
+papa|Tu la vois, la fourmi ?
+enfant-m|Oui.
+narrateur|La terre est sèche contre la peau.
+enfant-m|Elle pique, maman.
+maman|Tu la sens, la terre ?
+enfant-m|Oui.
+narrateur|Près du bord, un éclat de pot brille.
+enfant-m|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+narrateur|Une poussière danse au-dessus des pots.
+enfant-m|Elle vole, maman.
+maman|Au-dessus du bord ?
+enfant-m|Oui, au-dessus.
+narrateur|Papa pose les mains près de la terre.
+narrateur|La terre est un peu lourde.
+enfant-m|On fait le château, papa ?
+narrateur|Papa prend un peu de terre.
+narrateur|Un mur tombe un peu.
+enfant-m|C'est marron, papa.
+papa|Comme une maison ?
+enfant-m|Oui, comme une maison.
+narrateur|En ce moment, Victorino tire la terre vers les pots.
+enfant-m|Je veux le château, maintenant !
+enfant-m|Le château, tout de suite.
+papa|Tu vois la terre, Victorino ?
+enfant-m|Oui, papa.
+narrateur|Victorino ouvre les mains trop vite.
+narrateur|Il presse la terre trop fort.
+narrateur|Les murs collent trop près.
+enfant-m|Oh.
+narrateur|Le sourire de Victorino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Sa poitrine va trop vite.
+papa|Ça tombe, Victorino ?
+enfant-m|Oui, papa.
+maman|Tes lèvres sont serrées, Victorino ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de pot tremble, puis tient.
+narrateur|Le château s'effondre en tas.
+enfant-m|C'est trop, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Victorino regarde papa.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1404,17 +1416,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Le corps de Victorina va vite. Que fait-elle ?</t>
+          <t>Le corps de Victorino va vite. Que fait-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le corps de Victorina va vite. Que fait-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le corps de &lt;emphasis level="moderate"&gt;Victorino&lt;/emphasis&gt; va vite. Que fait-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le corps de William va vite. Que fait-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le corps de &lt;emphasis&gt;Victorino&lt;/emphasis&gt; va vite. Que fait-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1439,7 +1451,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Papa dit de souffler. Que fait William ensuite ?</t>
+          <t>Papa dit de souffler. Que fait Victorino ensuite ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1477,7 +1489,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1488,7 +1500,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1503,34 +1515,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Victorino</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1545,23 +1561,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_corps_va_vite_que_fait_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Le corps de Victorina va vite.
-narrateur|Que fait-elle ?</t>
+          <t>narrateur|Le corps de Victorino va vite.
+narrateur|Que fait-il ?</t>
         </is>
       </c>
     </row>
@@ -1588,17 +1604,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorina a soufflé. Elle a fait une pause. Son corps a ralenti. Le linge claque un peu, au vent. Tu as entendu le linge ? Oui. Il claque doucement. On reprend la terre, tout calme. Plus tard, un autre mur glisse un peu. Victorina sent encore sa poitrine. Je me souviens. Je souffle. Oui. Souffler, puis une pause. Elle s'assoit encore sur la planche. Le bois est chaud sous elle. Elle souffle. Elle fait une pause. Tes mains sont sur tes genoux. C'est bien. Tu as repris, tout calme. Le château est petit. Il tient.</t>
+          <t>Victorino veut le château, tout de suite. Je le fais, maintenant ! Il avance trop vite vers la terre. Les murs se referment, trop hauts. Victorino baisse les yeux. Sa poitrine est coincée. C'est trop. Victorino s'assoit près des pots. Victorino souffle, un filet d'air. Il reste un moment, sans bouger. Il fait une pause. Ses mains se ferment, puis s'ouvrent. Personne ne parle. Il observe les pots, un instant. Il écoute le silence du jardin. Tu veux le château avec la terre ? Papa reste à la même hauteur. Papa, on fait quoi ? Tu veux t'asseoir un peu ? D'accord. Victorino reste un moment, les mains ouvertes. Il souffle, plus long. La terre s'affaisse, puis tient. Merci, Victorino. Papa a vu le geste, au jardin. La terre est tiède, sous les doigts. Elle est chaude. Le mur tient, un peu de travers. Le château. Il a un toit, là ? Oui, là. Victorino glisse la main près du pot. La terre est douce, contre la peau. Tes mains sont au chaud, Victorino ? Un peu, maman. Papa pose un peu de terre. On le pose au bord ? Le château va jusqu'aux pots. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorina a soufflé. Elle a fait une pause. Son corps a ralenti. Le linge claque un peu, au vent. Tu as entendu le linge ? Oui. Il claque doucement. On reprend la terre, tout calme. Plus tard, un autre mur glisse un peu. Victorina sent encore sa poitrine. Je me souviens. Je souffle. Oui. Souffler, puis une pause. Elle s'assoit encore sur la planche. Le bois est chaud sous elle. Elle souffle. Elle fait une pause. Tes mains sont sur tes genoux. C'est bien. Tu as repris, tout calme. Le château est petit. Il tient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino veut le château, tout de suite. Je le fais, maintenant ! Il avance trop vite vers la terre. Les murs se referment, trop hauts. Victorino baisse les yeux. Sa poitrine est coincée. C'est trop. Victorino s'assoit près des pots. Victorino &lt;emphasis level="moderate"&gt;souffle&lt;/emphasis&gt;, un filet d'air. Il reste un moment, sans bouger. Il fait une pause. Ses mains se ferment, puis s'ouvrent. Personne ne parle. Il observe les pots, un instant. Il écoute le silence du jardin. Tu veux le château avec la terre ? Papa reste à la même hauteur. Papa, on fait quoi ? Tu veux t'asseoir un peu ? D'accord. Victorino reste un moment, les mains ouvertes. Il souffle, plus long. La terre s'affaisse, puis tient. Merci, Victorino. Papa a vu le geste, au jardin. La terre est tiède, sous les doigts. Elle est chaude. Le mur tient, un peu de travers. Le château. Il a un toit, là ? Oui, là. Victorino glisse la main près du pot. La terre est douce, contre la peau. Tes mains sont au chaud, Victorino ? Un peu, maman. Papa pose un peu de terre. On le pose au bord ? Le château va jusqu'aux pots. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>William a soufflé. Il a fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Son corps a ralenti. [pause]</t>
+          <t>Victorino veut le château, tout de suite. Je le fais, maintenant ! Il avance trop vite vers la terre. Les murs se referment, trop hauts. Victorino baisse les yeux. Sa poitrine est coincée. C'est trop. Victorino s'assoit près des pots. Victorino &lt;emphasis&gt;souffle&lt;/emphasis&gt;, un filet d'air. Il reste un moment, sans bouger. Il fait une pause. Ses mains se ferment, puis s'ouvrent. Personne ne parle. Il observe les pots, un instant. Il écoute le silence du jardin. Tu veux le château avec la terre ? Papa reste à la même hauteur. Papa, on fait quoi ? Tu veux t'asseoir un peu ? D'accord. Victorino reste un moment, les mains ouvertes. Il souffle, plus long. La terre s'affaisse, puis tient. Merci, Victorino. Papa a vu le geste, au jardin. La terre est tiède, sous les doigts. Elle est chaude. Le mur tient, un peu de travers. Le château. Il a un toit, là ? Oui, là. Victorino glisse la main près du pot. La terre est douce, contre la peau. Tes mains sont au chaud, Victorino ? Un peu, maman. Papa pose un peu de terre. On le pose au bord ? Le château va jusqu'aux pots. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1645,7 +1661,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1653,10 +1669,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1679,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>souffle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1711,10 +1727,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1727,29 +1743,50 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=gêne puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_souffle_il_fait_une_pause; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorina a soufflé.
-narrateur|Elle a fait une pause.
-narrateur|Son corps a ralenti.
-narrateur|Le linge claque un peu, au vent.
-maman|Tu as entendu le linge ?
-enfant-f|Oui. Il claque doucement.
-papa|On reprend la terre, tout calme.
-narrateur|Plus tard, un autre mur glisse un peu.
-narrateur|Victorina sent encore sa poitrine.
-enfant-f|Je me souviens. Je souffle.
-papa|Oui. Souffler, puis une pause.
-narrateur|Elle s'assoit encore sur la planche.
-narrateur|Le bois est chaud sous elle.
-narrateur|Elle souffle.
-narrateur|Elle fait une pause.
-maman|Tes mains sont sur tes genoux. C'est bien.
-papa|Tu as repris, tout calme.
-enfant-f|Le château est petit. Il tient.</t>
+          <t>narrateur|Victorino veut le château, tout de suite.
+enfant-m|Je le fais, maintenant !
+narrateur|Il avance trop vite vers la terre.
+narrateur|Les murs se referment, trop hauts.
+narrateur|Victorino baisse les yeux.
+narrateur|Sa poitrine est coincée.
+enfant-m|C'est trop.
+narrateur|Victorino s'assoit près des pots.
+narrateur|Victorino souffle, un filet d'air.
+narrateur|Il reste un moment, sans bouger.
+narrateur|Il fait une pause.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne parle.
+narrateur|Il observe les pots, un instant.
+narrateur|Il écoute le silence du jardin.
+papa|Tu veux le château avec la terre ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Papa, on fait quoi ?
+papa|Tu veux t'asseoir un peu ?
+enfant-m|D'accord.
+narrateur|Victorino reste un moment, les mains ouvertes.
+narrateur|Il souffle, plus long.
+narrateur|La terre s'affaisse, puis tient.
+papa|Merci, Victorino.
+narrateur|Papa a vu le geste, au jardin.
+maman|La terre est tiède, sous les doigts.
+enfant-m|Elle est chaude.
+narrateur|Le mur tient, un peu de travers.
+enfant-m|Le château.
+papa|Il a un toit, là ?
+enfant-m|Oui, là.
+narrateur|Victorino glisse la main près du pot.
+narrateur|La terre est douce, contre la peau.
+maman|Tes mains sont au chaud, Victorino ?
+enfant-m|Un peu, maman.
+narrateur|Papa pose un peu de terre.
+enfant-m|On le pose au bord ?
+maman|Le château va jusqu'aux pots.
+enfant-m|Oui, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1781,17 +1818,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Victorina ramasse une feuille. La feuille est verte et un peu rêche. Une toiture, papa. Tu la poses tout doux ? Elle pose la feuille sur le château. Le linge a séché. Vous voilà calmes. On range l'arrosoir ensemble ? Oui. Après le château. Le jardin sent encore la terre. Victorina essuie ses mains.</t>
+          <t>Ils restent près des pots. La terre tombe d'un côté. Le toit, maintenant ! Victorino presse la terre trop vite. Un pot penche vers le château. Ça glisse ! La terre cache un bout du mur. Victorino avance les mains, trop vite. Puis il s'arrête net. Il souffle, cette fois. Il fait une pause, plus longue. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le bord, un instant. Il écoute le silence du jardin. Au bord du pot, un éclat de pot luit. Là, sur le pot. Tu veux le château, papa ? Papa ne presse plus. Il tend les mains, sans presser. Je veux le château. Victorino pousse la terre, sans se presser. Papa la reçoit, plus loin. La terre est lisse et tiède. Tu le vois, le mur ? Oui, papa. Le château est près des pots ? Oui, maman. Papa pose un bord de terre. Victorino pose une main sur le pot. Le mur tient, Victorino ? Oui, papa. Un rayon passe sur le pot. Il allume la terre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Victorina ramasse une feuille. La feuille est verte et un peu rêche. Une toiture, papa. Tu la poses tout doux ? Elle pose la feuille sur le château. Le linge a séché. Vous voilà calmes. On range l'arrosoir ensemble ? Oui. Après le château. Le jardin sent encore la terre. Victorina essuie ses mains.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près des pots. La terre tombe d'un côté. Le toit, maintenant ! Victorino presse la terre trop vite. Un pot penche vers le château. Ça glisse ! La terre cache un bout du mur. Victorino avance les mains, trop vite. Puis il s'arrête net. Il souffle, cette fois. Il fait une pause, plus longue. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le bord, un instant. Il écoute le silence du jardin. Au bord du pot, un &lt;emphasis level="moderate"&gt;éclat de pot&lt;/emphasis&gt; luit. Là, sur le pot. Tu veux le château, papa ? Papa ne presse plus. Il tend les mains, sans presser. Je veux le château. Victorino pousse la terre, sans se presser. Papa la reçoit, plus loin. La terre est lisse et tiède. Tu le vois, le mur ? Oui, papa. Le château est près des pots ? Oui, maman. Papa pose un bord de terre. Victorino pose une main sur le pot. Le mur tient, Victorino ? Oui, papa. Un rayon passe sur le pot. Il allume la terre.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>William pose une feuille sur le château. Papa sourit. [pause]</t>
+          <t>Ils restent près des pots. La terre tombe d'un côté. Le toit, maintenant ! Victorino presse la terre trop vite. Un pot penche vers le château. Ça glisse ! La terre cache un bout du mur. Victorino avance les mains, trop vite. Puis il s'arrête net. Il souffle, cette fois. Il fait une pause, plus longue. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le bord, un instant. Il écoute le silence du jardin. Au bord du pot, un &lt;emphasis&gt;éclat de pot&lt;/emphasis&gt; luit. Là, sur le pot. Tu veux le château, papa ? Papa ne presse plus. Il tend les mains, sans presser. Je veux le château. Victorino pousse la terre, sans se presser. Papa la reçoit, plus loin. La terre est lisse et tiède. Tu le vois, le mur ? Oui, papa. Le château est près des pots ? Oui, maman. Papa pose un bord de terre. Victorino pose une main sur le pot. Le mur tient, Victorino ? Oui, papa. Un rayon passe sur le pot. Il allume la terre. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,7 +1875,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1846,10 +1883,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1870,28 +1907,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pot</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1900,10 +1941,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1914,24 +1955,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=pot_trop_vite_terre_glisse_il_souffle; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Victorina ramasse une feuille.
-narrateur|La feuille est verte et un peu rêche.
-enfant-f|Une toiture, papa.
-papa|Tu la poses tout doux ?
-narrateur|Elle pose la feuille sur le château.
-maman|Le linge a séché. Vous voilà calmes.
-papa|On range l'arrosoir ensemble ?
-enfant-f|Oui. Après le château.
-narrateur|Le jardin sent encore la terre.
-narrateur|Victorina essuie ses mains.</t>
+          <t>narrateur|Ils restent près des pots.
+narrateur|La terre tombe d'un côté.
+enfant-m|Le toit, maintenant !
+narrateur|Victorino presse la terre trop vite.
+narrateur|Un pot penche vers le château.
+enfant-m|Ça glisse !
+narrateur|La terre cache un bout du mur.
+narrateur|Victorino avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Il souffle, cette fois.
+narrateur|Il fait une pause, plus longue.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le bord, un instant.
+narrateur|Il écoute le silence du jardin.
+narrateur|Au bord du pot, un éclat de pot luit.
+enfant-m|Là, sur le pot.
+enfant-m|Tu veux le château, papa ?
+narrateur|Papa ne presse plus.
+narrateur|Il tend les mains, sans presser.
+papa|Je veux le château.
+narrateur|Victorino pousse la terre, sans se presser.
+narrateur|Papa la reçoit, plus loin.
+narrateur|La terre est lisse et tiède.
+papa|Tu le vois, le mur ?
+enfant-m|Oui, papa.
+maman|Le château est près des pots ?
+enfant-m|Oui, maman.
+narrateur|Papa pose un bord de terre.
+narrateur|Victorino pose une main sur le pot.
+papa|Le mur tient, Victorino ?
+enfant-m|Oui, papa.
+maman|Un rayon passe sur le pot.
+enfant-m|Il allume la terre.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>jardin,feuille</t>
+          <t>jardin,terre</t>
         </is>
       </c>
     </row>
@@ -1958,17 +2027,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Victorina. Le château a une feuille. Il est fini.</t>
+          <t>Ils restent près des pots. Le château est arrivé, Victorino ? Oui, maman. Tu souffles un peu ? Oui, papa. Victorino souffle, un filet d'air. La terre sent le basilic. Tu la sens, la terre ? Oui, maman. Le mur reste un peu, de travers. Il a tenu, près des pots. Le château. Le pot est chaud, sous les mains. L'ombre des pots fait un abri. On y retourne, après. Un éclat de pot tient sur la terre.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Victorina. Le château a une feuille. Il est fini.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près des pots. Le château est arrivé, Victorino ? Oui, maman. Tu souffles un peu ? Oui, papa. Victorino souffle, un filet d'air. La terre sent le basilic. Tu la sens, la terre ? Oui, maman. Le mur reste un peu, de travers. Il a tenu, près des pots. Le château. Le pot est chaud, sous les mains. L'ombre des pots fait un abri. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat de pot&lt;/emphasis&gt; tient sur la terre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près des pots. Le château est arrivé, Victorino ? Oui, maman. Tu souffles un peu ? Oui, papa. Victorino souffle, un filet d'air. La terre sent le basilic. Tu la sens, la terre ? Oui, maman. Le mur reste un peu, de travers. Il a tenu, près des pots. Le château. Le pot est chaud, sous les mains. L'ombre des pots fait un abri. On y retourne, après. Un &lt;emphasis&gt;éclat de pot&lt;/emphasis&gt; tient sur la terre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2015,7 +2084,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2023,10 +2092,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2035,12 +2104,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2049,17 +2118,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pot</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2068,11 +2141,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2081,26 +2154,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_terre; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai soufflé. J'ai fait une pause.
-papa|Bravo, Victorina.
-maman|Le château a une feuille. Il est fini.</t>
+          <t>narrateur|Ils restent près des pots.
+maman|Le château est arrivé, Victorino ?
+enfant-m|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-m|Oui, papa.
+narrateur|Victorino souffle, un filet d'air.
+enfant-m|La terre sent le basilic.
+maman|Tu la sens, la terre ?
+enfant-m|Oui, maman.
+papa|Le mur reste un peu, de travers.
+enfant-m|Il a tenu, près des pots.
+papa|Le château.
+narrateur|Le pot est chaud, sous les mains.
+narrateur|L'ombre des pots fait un abri.
+enfant-m|On y retourne, après.
+narrateur|Un éclat de pot tient sur la terre.</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2185,6 +2275,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>